<commit_message>
Milestone 2 - Java Support, AI Remediation, UI Polish, Gemini 2.5 Flash upgrades, Excel doc generation
</commit_message>
<xml_diff>
--- a/Agile_Template_v0.1.xlsx
+++ b/Agile_Template_v0.1.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -657,6 +657,158 @@
         </is>
       </c>
       <c r="H6" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B7" t="n">
+        <v>2</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>US03</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>As a developer, I want my code editor and results layout to be responsive and not vertically squished.</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Must Have</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>AI Agent</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>2</v>
+      </c>
+      <c r="B8" t="n">
+        <v>2</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>US04</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>As a developer, I want to automatically apply suggested code fixes directly to the editor.</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Must Have</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>US01</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>AI Agent</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>2</v>
+      </c>
+      <c r="B9" t="n">
+        <v>2</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>US05</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>As a user, I want the AI Assistant to provide context-aware chat about security findings.</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Must Have</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>US01</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>AI Agent</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>2</v>
+      </c>
+      <c r="B10" t="n">
+        <v>2</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>US06</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>As a user, I want to use the latest Gemini models for enhanced PR Summaries.</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Must Have</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>AI Agent</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
@@ -673,7 +825,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -735,6 +887,66 @@
       <c r="D3" t="inlineStr">
         <is>
           <t>Swapped localhost for 127.0.0.1 in Vite</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Day 13</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Gemini API 404 due to deprecated gemini-1.5-flash</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Updated backend to use gemini-flash-latest across all agents</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Day 14</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>UI Layout is squishing the Risk Score and right panel</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Replaced hardcoded grid with flex-wrap and 50/50 CSS Grid layout</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Day 15</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Apply Fix API returning 404</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Corrected frontend fetch route to point to /api/v1/submit/ prefix</t>
         </is>
       </c>
     </row>
@@ -749,7 +961,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -842,6 +1054,49 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="n">
+        <v>3</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>AI Agent</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Dynamically handling Gemini list responses</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Hardcoding LLM model versions</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Providing exact HTTP response mapping</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Implemented robust JSON &amp; String extraction for Gemini responses</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>